<commit_message>
Risorse 06-19 + Bonus + Indice rigenerate ad altissima qualità
- Stesso standard delle 01-05: brand AI Osha, no PMI, accenti corretti,
  footer Aliosha Battaglini + aiosha.it su ogni pagina, look del sito
- R06: NON più duplicato della R02 -> 12 scaffold riutilizzabili + 38 prompt avanzati
- R07/R10/R11/R16/R19: Excel con FORMULE funzionanti (dashboard, pipeline,
  P&L, valore pesato, budget totale, Gantt colorato, ROI business case)
- R08: corretta cifra free-tier Mailchimp; R09: 7 sezioni + esempio + prompt master
- R12: 20 prompt complementari a R02; R14: 12 workflow con tabella riepilogo
- R15: policy estesa coerente con R03; R17: checklist 4 settimane + tracker
- R18: guida NotebookLM step-by-step; Bonus: script video + versione breve
- 00_INDICE: rigenerato, mappa tutte le risorse ai capitoli
- Nomi file invariati: QR e link del libro restano validi

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risorse/Risorsa_07_Calendario_Editoriale.xlsx
+++ b/risorse/Risorsa_07_Calendario_Editoriale.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,25 +27,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A5F"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="0000838F"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -58,16 +51,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000BCD4"/>
+        <fgColor rgb="001E3A5F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000A1F2E"/>
+        <fgColor rgb="00E8F4FD"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -75,68 +68,29 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CFD8DC"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CFD8DC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CFD8DC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CFD8DC"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00C8E6C9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFF59D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFCDD2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -503,30 +457,30 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AIOsha · Risorsa 07 — Calendario Editoriale</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
+          <t>AI Osha — Risorsa 07 · Calendario Editoriale</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>30 giorni di contenuti pianificati con AI</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
+          <t>30 giorni di contenuti pianificati con l'AI. Aggiorna la colonna Stato: la Dashboard si calcola da sola.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Data</t>
@@ -601,7 +555,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>5 errori AI in PMI</t>
+          <t>5 errori con l'AI in azienda</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -609,55 +563,54 @@
           <t>Link in bio</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>02/05/2026</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Sab</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Instagram</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Mostrare lavoro</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Mostrare il lavoro</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Reel</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Caso reale: 4h risparmiate/sett</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Caso reale: 4h risparmiate a settimana</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -677,7 +630,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Fiducia/case study</t>
+          <t>Fiducia / case study</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -695,55 +648,54 @@
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>04/05/2026</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Lun</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Blog</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Vendere</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Newsletter</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Articolo</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Tool del mese + 3 prompt</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Link in bio</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -768,12 +720,12 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Blog</t>
+          <t>Carosello</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Guida completa: prompt per offerte</t>
+          <t>Guida: prompt per le offerte</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -781,55 +733,54 @@
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>06/05/2026</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Mer</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Instagram</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Mostrare lavoro</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Mostrare il lavoro</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Carosello</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Glossario AI in 7 termini</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -849,17 +800,17 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Fiducia/case study</t>
+          <t>Fiducia / case study</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Reel</t>
+          <t>Post testo</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Prima vs dopo AI in vendite</t>
+          <t>Prima vs dopo: AI nelle vendite</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -867,55 +818,54 @@
           <t>Link in bio</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>08/05/2026</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Ven</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Blog</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Vendere</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Carosello</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>5 errori AI in PMI</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Articolo</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>5 errori con l'AI in azienda</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -945,7 +895,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Caso reale: 4h risparmiate/sett</t>
+          <t>Caso reale: 4h risparmiate a settimana</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -953,55 +903,54 @@
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>10/05/2026</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Dom</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Instagram</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Mostrare lavoro</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Mostrare il lavoro</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>Post testo</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Cosa NON delegare all'AI</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Link in bio</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1021,12 +970,12 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Fiducia/case study</t>
+          <t>Fiducia / case study</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Newsletter</t>
+          <t>Post testo</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1039,55 +988,54 @@
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>12/05/2026</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Blog</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Vendere</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>Guida completa: prompt per offerte</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Articolo</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Guida: prompt per le offerte</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1125,55 +1073,54 @@
           <t>Link in bio</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>14/05/2026</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Gio</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Instagram</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Mostrare lavoro</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Mostrare il lavoro</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Reel</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>Prima vs dopo AI in vendite</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Prima vs dopo: AI nelle vendite</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1193,17 +1140,17 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Fiducia/case study</t>
+          <t>Fiducia / case study</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Carosello</t>
+          <t>Post testo</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>5 errori AI in PMI</t>
+          <t>5 errori con l'AI in azienda</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1211,55 +1158,54 @@
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>16/05/2026</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Sab</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Blog</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>Vendere</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Reel</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Caso reale: 4h risparmiate/sett</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Articolo</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Caso reale: 4h risparmiate a settimana</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>Link in bio</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1297,55 +1243,54 @@
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>18/05/2026</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Lun</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Instagram</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Mostrare lavoro</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Newsletter</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Mostrare il lavoro</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Carosello</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Tool del mese + 3 prompt</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr"/>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1365,73 +1310,72 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Fiducia/case study</t>
+          <t>Fiducia / case study</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
+          <t>Post testo</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Guida: prompt per le offerte</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Link in bio</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Mer</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
           <t>Blog</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Guida completa: prompt per offerte</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Link in bio</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Mer</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>Vendere</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Carosello</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Articolo</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>Glossario AI in 7 termini</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1461,7 +1405,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Prima vs dopo AI in vendite</t>
+          <t>Prima vs dopo: AI nelle vendite</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1469,55 +1413,54 @@
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>22/05/2026</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Ven</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Instagram</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Mostrare lavoro</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Mostrare il lavoro</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Carosello</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>5 errori AI in PMI</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>5 errori con l'AI in azienda</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>Link in bio</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I26" s="4" t="inlineStr"/>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1537,17 +1480,17 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Fiducia/case study</t>
+          <t>Fiducia / case study</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Reel</t>
+          <t>Post testo</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Caso reale: 4h risparmiate/sett</t>
+          <t>Caso reale: 4h risparmiate a settimana</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1555,55 +1498,54 @@
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>24/05/2026</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Dom</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Blog</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>Vendere</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>Post testo</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Articolo</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>Cosa NON delegare all'AI</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr"/>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1628,7 +1570,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Newsletter</t>
+          <t>Carosello</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1641,55 +1583,54 @@
           <t>Link in bio</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>26/05/2026</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Instagram</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>Mostrare lavoro</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>Guida completa: prompt per offerte</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Mostrare il lavoro</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Guida: prompt per le offerte</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I30" s="4" t="inlineStr"/>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1709,12 +1650,12 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Fiducia/case study</t>
+          <t>Fiducia / case study</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Carosello</t>
+          <t>Post testo</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -1727,55 +1668,54 @@
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I31" s="4" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>28/05/2026</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>Gio</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>Blog</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>Vendere</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Reel</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>Prima vs dopo AI in vendite</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Articolo</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Prima vs dopo: AI nelle vendite</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>Link in bio</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I32" s="4" t="inlineStr"/>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -1805,7 +1745,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>5 errori AI in PMI</t>
+          <t>5 errori con l'AI in azienda</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1813,72 +1753,61 @@
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>30/05/2026</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>Sab</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>Instagram</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Mostrare lavoro</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Mostrare il lavoro</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>Reel</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>Caso reale: 4h risparmiate/sett</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Caso reale: 4h risparmiate a settimana</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>Commenta</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr"/>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-  </mergeCells>
-  <conditionalFormatting sqref="H5:H34">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"Pubblicato"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
-      <formula>"In bozza"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
-      <formula>"Da fare"</formula>
-    </cfRule>
-  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Da fare,In bozza,Pubblicato"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1889,24 +1818,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AIOsha · Dashboard mese</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
+          <t>AI Osha — Dashboard del mese</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Metriche di pubblicazione</t>
+          <t>Si aggiorna in automatico dai dati del foglio Calendario.</t>
         </is>
       </c>
     </row>
@@ -1923,109 +1852,105 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Totale post pianificati</t>
         </is>
       </c>
-      <c r="B5" s="4">
+      <c r="B5">
         <f>COUNTA(Calendario!F5:F34)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Pubblicati</t>
         </is>
       </c>
-      <c r="B6" s="4">
+      <c r="B6">
         <f>COUNTIF(Calendario!H5:H34,"Pubblicato")</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>In bozza</t>
         </is>
       </c>
-      <c r="B7" s="4">
+      <c r="B7">
         <f>COUNTIF(Calendario!H5:H34,"In bozza")</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="B8" s="4">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="B8">
         <f>COUNTIF(Calendario!H5:H34,"Da fare")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>% completato</t>
         </is>
       </c>
-      <c r="B9" s="5">
-        <f>IFERROR(B6/B5,0)</f>
+      <c r="B9" s="7">
+        <f>IF(B5=0,0,B6/B5)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="B10" s="4">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Post LinkedIn</t>
+        </is>
+      </c>
+      <c r="B10">
         <f>COUNTIF(Calendario!C5:C34,"LinkedIn")</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="B11" s="4">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Post Instagram</t>
+        </is>
+      </c>
+      <c r="B11">
         <f>COUNTIF(Calendario!C5:C34,"Instagram")</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Newsletter</t>
-        </is>
-      </c>
-      <c r="B12" s="4">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Post Newsletter</t>
+        </is>
+      </c>
+      <c r="B12">
         <f>COUNTIF(Calendario!C5:C34,"Newsletter")</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="B13" s="4">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Post Blog</t>
+        </is>
+      </c>
+      <c r="B13">
         <f>COUNTIF(Calendario!C5:C34,"Blog")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>